<commit_message>
Offhands kalibriert: Prim 3/5/7/10/14/18/24, Kapazität = Stufe, Verfeinerung 1/2/3+ (inkl. Stufe 7)
- offhands.json v1.3: alle 84 Einträge mit kalibrierten Prim.-Werten (= Sekundärslot-Tier, ~50% des Zweihand-Äquivalents) und Max. Verfeinerung analog Waffen; Stellar ausgearbeitet
- itemliste_v7.xlsx: Offhands-Sheet neu generiert und gegen JSON verifiziert
- GDD §5.3: Werte-Tabelle + Begründung; §5.7: Slot-Beispiel ergänzt (Kapazität 1 + Aktiv-Slot); §11 Phase-0-Punkt 1 abgehakt; GDD v0.13
- CLAUDE.md: Sitzungsstand, Kurzreferenz, nächste Schritte

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017YKvWczRrwfVjxabHvNySm
</commit_message>
<xml_diff>
--- a/data/itemliste_v7.xlsx
+++ b/data/itemliste_v7.xlsx
@@ -31559,7 +31559,7 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -31655,7 +31655,7 @@
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -31751,7 +31751,7 @@
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -31839,7 +31839,7 @@
         <v>4</v>
       </c>
       <c r="O6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -31847,7 +31847,7 @@
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -31935,7 +31935,7 @@
         <v>5</v>
       </c>
       <c r="O7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -31943,7 +31943,7 @@
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -32031,7 +32031,7 @@
         <v>6</v>
       </c>
       <c r="O8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -32039,7 +32039,7 @@
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -32127,7 +32127,7 @@
         <v>7</v>
       </c>
       <c r="O9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -32135,7 +32135,7 @@
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -32150,6 +32150,11 @@
       <c r="T9" t="inlineStr">
         <is>
           <t>Schildbuckel</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V9" t="n">
@@ -32256,7 +32261,7 @@
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -32352,7 +32357,7 @@
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -32448,7 +32453,7 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -32536,7 +32541,7 @@
         <v>4</v>
       </c>
       <c r="O14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
@@ -32544,7 +32549,7 @@
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -32632,7 +32637,7 @@
         <v>5</v>
       </c>
       <c r="O15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
@@ -32640,7 +32645,7 @@
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -32728,7 +32733,7 @@
         <v>6</v>
       </c>
       <c r="O16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
@@ -32736,7 +32741,7 @@
         </is>
       </c>
       <c r="Q16" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -32824,7 +32829,7 @@
         <v>7</v>
       </c>
       <c r="O17" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
@@ -32832,7 +32837,7 @@
         </is>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -32847,6 +32852,11 @@
       <c r="T17" t="inlineStr">
         <is>
           <t>Großschild + Stützarm</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V17" t="n">
@@ -32953,7 +32963,7 @@
         </is>
       </c>
       <c r="Q19" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -33049,7 +33059,7 @@
         </is>
       </c>
       <c r="Q20" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
@@ -33145,7 +33155,7 @@
         </is>
       </c>
       <c r="Q21" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
@@ -33233,7 +33243,7 @@
         <v>4</v>
       </c>
       <c r="O22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
@@ -33241,7 +33251,7 @@
         </is>
       </c>
       <c r="Q22" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -33329,7 +33339,7 @@
         <v>5</v>
       </c>
       <c r="O23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
@@ -33337,7 +33347,7 @@
         </is>
       </c>
       <c r="Q23" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
@@ -33425,7 +33435,7 @@
         <v>6</v>
       </c>
       <c r="O24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
@@ -33433,7 +33443,7 @@
         </is>
       </c>
       <c r="Q24" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
@@ -33521,7 +33531,7 @@
         <v>7</v>
       </c>
       <c r="O25" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
@@ -33529,7 +33539,7 @@
         </is>
       </c>
       <c r="Q25" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
@@ -33544,6 +33554,11 @@
       <c r="T25" t="inlineStr">
         <is>
           <t>Einband + Seiten</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V25" t="n">
@@ -33650,7 +33665,7 @@
         </is>
       </c>
       <c r="Q27" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
@@ -33746,7 +33761,7 @@
         </is>
       </c>
       <c r="Q28" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
@@ -33842,7 +33857,7 @@
         </is>
       </c>
       <c r="Q29" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
@@ -33930,7 +33945,7 @@
         <v>4</v>
       </c>
       <c r="O30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
@@ -33938,7 +33953,7 @@
         </is>
       </c>
       <c r="Q30" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -34026,7 +34041,7 @@
         <v>5</v>
       </c>
       <c r="O31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
@@ -34034,7 +34049,7 @@
         </is>
       </c>
       <c r="Q31" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
@@ -34122,7 +34137,7 @@
         <v>6</v>
       </c>
       <c r="O32" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
@@ -34130,7 +34145,7 @@
         </is>
       </c>
       <c r="Q32" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
@@ -34218,7 +34233,7 @@
         <v>7</v>
       </c>
       <c r="O33" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
@@ -34226,7 +34241,7 @@
         </is>
       </c>
       <c r="Q33" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
@@ -34241,6 +34256,11 @@
       <c r="T33" t="inlineStr">
         <is>
           <t>Geschliffener Kristall</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V33" t="n">
@@ -34347,7 +34367,7 @@
         </is>
       </c>
       <c r="Q35" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
@@ -34443,7 +34463,7 @@
         </is>
       </c>
       <c r="Q36" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
@@ -34539,7 +34559,7 @@
         </is>
       </c>
       <c r="Q37" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
@@ -34627,7 +34647,7 @@
         <v>4</v>
       </c>
       <c r="O38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
@@ -34635,7 +34655,7 @@
         </is>
       </c>
       <c r="Q38" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
@@ -34723,7 +34743,7 @@
         <v>5</v>
       </c>
       <c r="O39" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P39" t="inlineStr">
         <is>
@@ -34731,7 +34751,7 @@
         </is>
       </c>
       <c r="Q39" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
@@ -34819,7 +34839,7 @@
         <v>6</v>
       </c>
       <c r="O40" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P40" t="inlineStr">
         <is>
@@ -34827,7 +34847,7 @@
         </is>
       </c>
       <c r="Q40" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
@@ -34915,7 +34935,7 @@
         <v>7</v>
       </c>
       <c r="O41" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P41" t="inlineStr">
         <is>
@@ -34923,7 +34943,7 @@
         </is>
       </c>
       <c r="Q41" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
@@ -34938,6 +34958,11 @@
       <c r="T41" t="inlineStr">
         <is>
           <t>Kette + Griffring</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V41" t="n">
@@ -35044,7 +35069,7 @@
         </is>
       </c>
       <c r="Q43" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
@@ -35140,7 +35165,7 @@
         </is>
       </c>
       <c r="Q44" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
@@ -35236,7 +35261,7 @@
         </is>
       </c>
       <c r="Q45" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
@@ -35324,7 +35349,7 @@
         <v>4</v>
       </c>
       <c r="O46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P46" t="inlineStr">
         <is>
@@ -35332,7 +35357,7 @@
         </is>
       </c>
       <c r="Q46" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
@@ -35420,7 +35445,7 @@
         <v>5</v>
       </c>
       <c r="O47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P47" t="inlineStr">
         <is>
@@ -35428,7 +35453,7 @@
         </is>
       </c>
       <c r="Q47" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
@@ -35516,7 +35541,7 @@
         <v>6</v>
       </c>
       <c r="O48" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P48" t="inlineStr">
         <is>
@@ -35524,7 +35549,7 @@
         </is>
       </c>
       <c r="Q48" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
@@ -35612,7 +35637,7 @@
         <v>7</v>
       </c>
       <c r="O49" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P49" t="inlineStr">
         <is>
@@ -35620,7 +35645,7 @@
         </is>
       </c>
       <c r="Q49" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
@@ -35635,6 +35660,11 @@
       <c r="T49" t="inlineStr">
         <is>
           <t>Gehäuse + Glas</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V49" t="n">
@@ -35741,7 +35771,7 @@
         </is>
       </c>
       <c r="Q51" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
@@ -35837,7 +35867,7 @@
         </is>
       </c>
       <c r="Q52" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
@@ -35933,7 +35963,7 @@
         </is>
       </c>
       <c r="Q53" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
@@ -36021,7 +36051,7 @@
         <v>4</v>
       </c>
       <c r="O54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P54" t="inlineStr">
         <is>
@@ -36029,7 +36059,7 @@
         </is>
       </c>
       <c r="Q54" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R54" t="inlineStr">
         <is>
@@ -36117,7 +36147,7 @@
         <v>5</v>
       </c>
       <c r="O55" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P55" t="inlineStr">
         <is>
@@ -36125,7 +36155,7 @@
         </is>
       </c>
       <c r="Q55" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
@@ -36213,7 +36243,7 @@
         <v>6</v>
       </c>
       <c r="O56" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P56" t="inlineStr">
         <is>
@@ -36221,7 +36251,7 @@
         </is>
       </c>
       <c r="Q56" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
@@ -36309,7 +36339,7 @@
         <v>7</v>
       </c>
       <c r="O57" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P57" t="inlineStr">
         <is>
@@ -36317,7 +36347,7 @@
         </is>
       </c>
       <c r="Q57" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
@@ -36332,6 +36362,11 @@
       <c r="T57" t="inlineStr">
         <is>
           <t>Gurt + Schnalle</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V57" t="n">
@@ -36438,7 +36473,7 @@
         </is>
       </c>
       <c r="Q59" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
@@ -36534,7 +36569,7 @@
         </is>
       </c>
       <c r="Q60" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
@@ -36630,7 +36665,7 @@
         </is>
       </c>
       <c r="Q61" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R61" t="inlineStr">
         <is>
@@ -36718,7 +36753,7 @@
         <v>4</v>
       </c>
       <c r="O62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P62" t="inlineStr">
         <is>
@@ -36726,7 +36761,7 @@
         </is>
       </c>
       <c r="Q62" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R62" t="inlineStr">
         <is>
@@ -36814,7 +36849,7 @@
         <v>5</v>
       </c>
       <c r="O63" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P63" t="inlineStr">
         <is>
@@ -36822,7 +36857,7 @@
         </is>
       </c>
       <c r="Q63" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R63" t="inlineStr">
         <is>
@@ -36910,7 +36945,7 @@
         <v>6</v>
       </c>
       <c r="O64" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P64" t="inlineStr">
         <is>
@@ -36918,7 +36953,7 @@
         </is>
       </c>
       <c r="Q64" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R64" t="inlineStr">
         <is>
@@ -37006,7 +37041,7 @@
         <v>7</v>
       </c>
       <c r="O65" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P65" t="inlineStr">
         <is>
@@ -37014,7 +37049,7 @@
         </is>
       </c>
       <c r="Q65" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
@@ -37029,6 +37064,11 @@
       <c r="T65" t="inlineStr">
         <is>
           <t>Schaft + Pechkopf</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V65" t="n">
@@ -37135,7 +37175,7 @@
         </is>
       </c>
       <c r="Q67" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
@@ -37231,7 +37271,7 @@
         </is>
       </c>
       <c r="Q68" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
@@ -37327,7 +37367,7 @@
         </is>
       </c>
       <c r="Q69" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
@@ -37415,7 +37455,7 @@
         <v>4</v>
       </c>
       <c r="O70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P70" t="inlineStr">
         <is>
@@ -37423,7 +37463,7 @@
         </is>
       </c>
       <c r="Q70" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
@@ -37511,7 +37551,7 @@
         <v>5</v>
       </c>
       <c r="O71" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P71" t="inlineStr">
         <is>
@@ -37519,7 +37559,7 @@
         </is>
       </c>
       <c r="Q71" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R71" t="inlineStr">
         <is>
@@ -37607,7 +37647,7 @@
         <v>6</v>
       </c>
       <c r="O72" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P72" t="inlineStr">
         <is>
@@ -37615,7 +37655,7 @@
         </is>
       </c>
       <c r="Q72" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R72" t="inlineStr">
         <is>
@@ -37703,7 +37743,7 @@
         <v>7</v>
       </c>
       <c r="O73" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P73" t="inlineStr">
         <is>
@@ -37711,7 +37751,7 @@
         </is>
       </c>
       <c r="Q73" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R73" t="inlineStr">
         <is>
@@ -37726,6 +37766,11 @@
       <c r="T73" t="inlineStr">
         <is>
           <t>Horn + Mundstück</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V73" t="n">
@@ -37832,7 +37877,7 @@
         </is>
       </c>
       <c r="Q75" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R75" t="inlineStr">
         <is>
@@ -37928,7 +37973,7 @@
         </is>
       </c>
       <c r="Q76" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R76" t="inlineStr">
         <is>
@@ -38024,7 +38069,7 @@
         </is>
       </c>
       <c r="Q77" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R77" t="inlineStr">
         <is>
@@ -38112,7 +38157,7 @@
         <v>4</v>
       </c>
       <c r="O78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P78" t="inlineStr">
         <is>
@@ -38120,7 +38165,7 @@
         </is>
       </c>
       <c r="Q78" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R78" t="inlineStr">
         <is>
@@ -38208,7 +38253,7 @@
         <v>5</v>
       </c>
       <c r="O79" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P79" t="inlineStr">
         <is>
@@ -38216,7 +38261,7 @@
         </is>
       </c>
       <c r="Q79" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R79" t="inlineStr">
         <is>
@@ -38304,7 +38349,7 @@
         <v>6</v>
       </c>
       <c r="O80" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P80" t="inlineStr">
         <is>
@@ -38312,7 +38357,7 @@
         </is>
       </c>
       <c r="Q80" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R80" t="inlineStr">
         <is>
@@ -38400,7 +38445,7 @@
         <v>7</v>
       </c>
       <c r="O81" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P81" t="inlineStr">
         <is>
@@ -38408,7 +38453,7 @@
         </is>
       </c>
       <c r="Q81" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R81" t="inlineStr">
         <is>
@@ -38423,6 +38468,11 @@
       <c r="T81" t="inlineStr">
         <is>
           <t>Stange + Banner</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V81" t="n">
@@ -38529,7 +38579,7 @@
         </is>
       </c>
       <c r="Q83" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R83" t="inlineStr">
         <is>
@@ -38625,7 +38675,7 @@
         </is>
       </c>
       <c r="Q84" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R84" t="inlineStr">
         <is>
@@ -38721,7 +38771,7 @@
         </is>
       </c>
       <c r="Q85" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R85" t="inlineStr">
         <is>
@@ -38809,7 +38859,7 @@
         <v>4</v>
       </c>
       <c r="O86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P86" t="inlineStr">
         <is>
@@ -38817,7 +38867,7 @@
         </is>
       </c>
       <c r="Q86" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R86" t="inlineStr">
         <is>
@@ -38905,7 +38955,7 @@
         <v>5</v>
       </c>
       <c r="O87" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P87" t="inlineStr">
         <is>
@@ -38913,7 +38963,7 @@
         </is>
       </c>
       <c r="Q87" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R87" t="inlineStr">
         <is>
@@ -39001,7 +39051,7 @@
         <v>6</v>
       </c>
       <c r="O88" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P88" t="inlineStr">
         <is>
@@ -39009,7 +39059,7 @@
         </is>
       </c>
       <c r="Q88" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R88" t="inlineStr">
         <is>
@@ -39097,7 +39147,7 @@
         <v>7</v>
       </c>
       <c r="O89" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P89" t="inlineStr">
         <is>
@@ -39105,7 +39155,7 @@
         </is>
       </c>
       <c r="Q89" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R89" t="inlineStr">
         <is>
@@ -39120,6 +39170,11 @@
       <c r="T89" t="inlineStr">
         <is>
           <t>Gefäß + Kette</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V89" t="n">
@@ -39226,7 +39281,7 @@
         </is>
       </c>
       <c r="Q91" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R91" t="inlineStr">
         <is>
@@ -39322,7 +39377,7 @@
         </is>
       </c>
       <c r="Q92" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="R92" t="inlineStr">
         <is>
@@ -39418,7 +39473,7 @@
         </is>
       </c>
       <c r="Q93" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="R93" t="inlineStr">
         <is>
@@ -39506,7 +39561,7 @@
         <v>4</v>
       </c>
       <c r="O94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P94" t="inlineStr">
         <is>
@@ -39514,7 +39569,7 @@
         </is>
       </c>
       <c r="Q94" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R94" t="inlineStr">
         <is>
@@ -39602,7 +39657,7 @@
         <v>5</v>
       </c>
       <c r="O95" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P95" t="inlineStr">
         <is>
@@ -39610,7 +39665,7 @@
         </is>
       </c>
       <c r="Q95" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="R95" t="inlineStr">
         <is>
@@ -39698,7 +39753,7 @@
         <v>6</v>
       </c>
       <c r="O96" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P96" t="inlineStr">
         <is>
@@ -39706,7 +39761,7 @@
         </is>
       </c>
       <c r="Q96" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R96" t="inlineStr">
         <is>
@@ -39794,7 +39849,7 @@
         <v>7</v>
       </c>
       <c r="O97" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P97" t="inlineStr">
         <is>
@@ -39802,7 +39857,7 @@
         </is>
       </c>
       <c r="Q97" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="R97" t="inlineStr">
         <is>
@@ -39817,6 +39872,11 @@
       <c r="T97" t="inlineStr">
         <is>
           <t>Kolben + Lockstoff</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="V97" t="n">

</xml_diff>

<commit_message>
Rüstung: Max. Verfeinerung auf 1×/2×/3×-Modell korrigiert, Slot-Kapazitäten final
- Kopf-/Körper-/Fußausrüstung (je v1.2): Max. Verfeinerung war versehentlich = Stufe
  (bis 7×) — korrigiert auf 1× Kupfer / 2× Eisen / 3× ab Stahl, wie Waffen/Offhands
  (84 Einträge, inkl. Zubehör)
- Slot-Kapazitäten bestätigt: Grundkapazität = Stufe, Slots 1 bis Stahl / 2 ab Titan
- verfeinerungs_regel in stat_skalierung ergänzt, meta.status aktualisiert
- itemliste_v7.xlsx: drei Rüstungs-Sheets angeglichen
- GDD §11: Checklisten-Punkte annotiert

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LMPve8W3NYqANspaTmaDDr
</commit_message>
<xml_diff>
--- a/data/itemliste_v7.xlsx
+++ b/data/itemliste_v7.xlsx
@@ -1309,7 +1309,7 @@
         <v>4</v>
       </c>
       <c r="O6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P6" t="n">
         <v>8</v>
@@ -1417,7 +1417,7 @@
         <v>5</v>
       </c>
       <c r="O7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P7" t="n">
         <v>10</v>
@@ -1525,7 +1525,7 @@
         <v>6</v>
       </c>
       <c r="O8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P8" t="n">
         <v>14</v>
@@ -1633,7 +1633,7 @@
         <v>7</v>
       </c>
       <c r="O9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -2094,7 +2094,7 @@
         <v>4</v>
       </c>
       <c r="O14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P14" t="n">
         <v>8</v>
@@ -2202,7 +2202,7 @@
         <v>5</v>
       </c>
       <c r="O15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P15" t="n">
         <v>10</v>
@@ -2310,7 +2310,7 @@
         <v>6</v>
       </c>
       <c r="O16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P16" t="n">
         <v>14</v>
@@ -2418,7 +2418,7 @@
         <v>7</v>
       </c>
       <c r="O17" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
@@ -2879,7 +2879,7 @@
         <v>4</v>
       </c>
       <c r="O22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P22" t="n">
         <v>10</v>
@@ -2987,7 +2987,7 @@
         <v>5</v>
       </c>
       <c r="O23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P23" t="n">
         <v>13</v>
@@ -3095,7 +3095,7 @@
         <v>6</v>
       </c>
       <c r="O24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P24" t="n">
         <v>17</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="O25" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
@@ -3664,7 +3664,7 @@
         <v>4</v>
       </c>
       <c r="O30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P30" t="n">
         <v>10</v>
@@ -3772,7 +3772,7 @@
         <v>5</v>
       </c>
       <c r="O31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P31" t="n">
         <v>13</v>
@@ -3880,7 +3880,7 @@
         <v>6</v>
       </c>
       <c r="O32" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P32" t="n">
         <v>17</v>
@@ -3988,7 +3988,7 @@
         <v>7</v>
       </c>
       <c r="O33" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
@@ -4449,7 +4449,7 @@
         <v>4</v>
       </c>
       <c r="O38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P38" t="n">
         <v>14</v>
@@ -4557,7 +4557,7 @@
         <v>5</v>
       </c>
       <c r="O39" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P39" t="n">
         <v>18</v>
@@ -4665,7 +4665,7 @@
         <v>6</v>
       </c>
       <c r="O40" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P40" t="n">
         <v>24</v>
@@ -4773,7 +4773,7 @@
         <v>7</v>
       </c>
       <c r="O41" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P41" t="n">
         <v>0</v>
@@ -5234,7 +5234,7 @@
         <v>4</v>
       </c>
       <c r="O46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P46" t="n">
         <v>0</v>
@@ -5342,7 +5342,7 @@
         <v>5</v>
       </c>
       <c r="O47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P47" t="n">
         <v>0</v>
@@ -5450,7 +5450,7 @@
         <v>6</v>
       </c>
       <c r="O48" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P48" t="n">
         <v>0</v>
@@ -5558,7 +5558,7 @@
         <v>7</v>
       </c>
       <c r="O49" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P49" t="n">
         <v>0</v>
@@ -6019,7 +6019,7 @@
         <v>4</v>
       </c>
       <c r="O54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P54" t="n">
         <v>0</v>
@@ -6127,7 +6127,7 @@
         <v>5</v>
       </c>
       <c r="O55" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P55" t="n">
         <v>0</v>
@@ -6235,7 +6235,7 @@
         <v>6</v>
       </c>
       <c r="O56" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P56" t="n">
         <v>0</v>
@@ -6343,7 +6343,7 @@
         <v>7</v>
       </c>
       <c r="O57" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P57" t="n">
         <v>0</v>
@@ -6994,7 +6994,7 @@
         <v>4</v>
       </c>
       <c r="O6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P6" t="n">
         <v>5</v>
@@ -7105,7 +7105,7 @@
         <v>5</v>
       </c>
       <c r="O7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P7" t="n">
         <v>6</v>
@@ -7216,7 +7216,7 @@
         <v>6</v>
       </c>
       <c r="O8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P8" t="n">
         <v>8</v>
@@ -7327,7 +7327,7 @@
         <v>7</v>
       </c>
       <c r="O9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -7801,7 +7801,7 @@
         <v>4</v>
       </c>
       <c r="O14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P14" t="n">
         <v>5</v>
@@ -7912,7 +7912,7 @@
         <v>5</v>
       </c>
       <c r="O15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P15" t="n">
         <v>6</v>
@@ -8023,7 +8023,7 @@
         <v>6</v>
       </c>
       <c r="O16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P16" t="n">
         <v>8</v>
@@ -8134,7 +8134,7 @@
         <v>7</v>
       </c>
       <c r="O17" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
@@ -8608,7 +8608,7 @@
         <v>4</v>
       </c>
       <c r="O22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P22" t="n">
         <v>6</v>
@@ -8719,7 +8719,7 @@
         <v>5</v>
       </c>
       <c r="O23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P23" t="n">
         <v>8</v>
@@ -8830,7 +8830,7 @@
         <v>6</v>
       </c>
       <c r="O24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P24" t="n">
         <v>10</v>
@@ -8941,7 +8941,7 @@
         <v>7</v>
       </c>
       <c r="O25" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
@@ -9415,7 +9415,7 @@
         <v>4</v>
       </c>
       <c r="O30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P30" t="n">
         <v>6</v>
@@ -9526,7 +9526,7 @@
         <v>5</v>
       </c>
       <c r="O31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P31" t="n">
         <v>8</v>
@@ -9637,7 +9637,7 @@
         <v>6</v>
       </c>
       <c r="O32" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P32" t="n">
         <v>10</v>
@@ -9748,7 +9748,7 @@
         <v>7</v>
       </c>
       <c r="O33" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
@@ -10222,7 +10222,7 @@
         <v>4</v>
       </c>
       <c r="O38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P38" t="n">
         <v>8</v>
@@ -10333,7 +10333,7 @@
         <v>5</v>
       </c>
       <c r="O39" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P39" t="n">
         <v>11</v>
@@ -10444,7 +10444,7 @@
         <v>6</v>
       </c>
       <c r="O40" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P40" t="n">
         <v>14</v>
@@ -10555,7 +10555,7 @@
         <v>7</v>
       </c>
       <c r="O41" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P41" t="n">
         <v>0</v>
@@ -11029,7 +11029,7 @@
         <v>4</v>
       </c>
       <c r="O46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P46" t="n">
         <v>0</v>
@@ -11140,7 +11140,7 @@
         <v>5</v>
       </c>
       <c r="O47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P47" t="n">
         <v>0</v>
@@ -11251,7 +11251,7 @@
         <v>6</v>
       </c>
       <c r="O48" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P48" t="n">
         <v>0</v>
@@ -11362,7 +11362,7 @@
         <v>7</v>
       </c>
       <c r="O49" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P49" t="n">
         <v>0</v>
@@ -11836,7 +11836,7 @@
         <v>4</v>
       </c>
       <c r="O54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P54" t="n">
         <v>0</v>
@@ -11947,7 +11947,7 @@
         <v>5</v>
       </c>
       <c r="O55" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P55" t="n">
         <v>0</v>
@@ -12058,7 +12058,7 @@
         <v>6</v>
       </c>
       <c r="O56" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P56" t="n">
         <v>0</v>
@@ -12169,7 +12169,7 @@
         <v>7</v>
       </c>
       <c r="O57" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P57" t="n">
         <v>0</v>
@@ -40477,7 +40477,7 @@
         <v>4</v>
       </c>
       <c r="O6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P6" t="n">
         <v>5</v>
@@ -40585,7 +40585,7 @@
         <v>5</v>
       </c>
       <c r="O7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P7" t="n">
         <v>6</v>
@@ -40693,7 +40693,7 @@
         <v>6</v>
       </c>
       <c r="O8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P8" t="n">
         <v>8</v>
@@ -40801,7 +40801,7 @@
         <v>7</v>
       </c>
       <c r="O9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -41262,7 +41262,7 @@
         <v>4</v>
       </c>
       <c r="O14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P14" t="n">
         <v>5</v>
@@ -41370,7 +41370,7 @@
         <v>5</v>
       </c>
       <c r="O15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P15" t="n">
         <v>6</v>
@@ -41478,7 +41478,7 @@
         <v>6</v>
       </c>
       <c r="O16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P16" t="n">
         <v>8</v>
@@ -41586,7 +41586,7 @@
         <v>7</v>
       </c>
       <c r="O17" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
@@ -42047,7 +42047,7 @@
         <v>4</v>
       </c>
       <c r="O22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P22" t="n">
         <v>6</v>
@@ -42155,7 +42155,7 @@
         <v>5</v>
       </c>
       <c r="O23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P23" t="n">
         <v>8</v>
@@ -42263,7 +42263,7 @@
         <v>6</v>
       </c>
       <c r="O24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P24" t="n">
         <v>10</v>
@@ -42371,7 +42371,7 @@
         <v>7</v>
       </c>
       <c r="O25" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
@@ -42832,7 +42832,7 @@
         <v>4</v>
       </c>
       <c r="O30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P30" t="n">
         <v>6</v>
@@ -42940,7 +42940,7 @@
         <v>5</v>
       </c>
       <c r="O31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P31" t="n">
         <v>8</v>
@@ -43048,7 +43048,7 @@
         <v>6</v>
       </c>
       <c r="O32" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P32" t="n">
         <v>10</v>
@@ -43156,7 +43156,7 @@
         <v>7</v>
       </c>
       <c r="O33" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
@@ -43617,7 +43617,7 @@
         <v>4</v>
       </c>
       <c r="O38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P38" t="n">
         <v>8</v>
@@ -43725,7 +43725,7 @@
         <v>5</v>
       </c>
       <c r="O39" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P39" t="n">
         <v>11</v>
@@ -43833,7 +43833,7 @@
         <v>6</v>
       </c>
       <c r="O40" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P40" t="n">
         <v>14</v>
@@ -43941,7 +43941,7 @@
         <v>7</v>
       </c>
       <c r="O41" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P41" t="n">
         <v>0</v>
@@ -44402,7 +44402,7 @@
         <v>4</v>
       </c>
       <c r="O46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P46" t="n">
         <v>0</v>
@@ -44510,7 +44510,7 @@
         <v>5</v>
       </c>
       <c r="O47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P47" t="n">
         <v>0</v>
@@ -44618,7 +44618,7 @@
         <v>6</v>
       </c>
       <c r="O48" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P48" t="n">
         <v>0</v>
@@ -44726,7 +44726,7 @@
         <v>7</v>
       </c>
       <c r="O49" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P49" t="n">
         <v>0</v>
@@ -45187,7 +45187,7 @@
         <v>4</v>
       </c>
       <c r="O54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P54" t="n">
         <v>0</v>
@@ -45295,7 +45295,7 @@
         <v>5</v>
       </c>
       <c r="O55" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P55" t="n">
         <v>0</v>
@@ -45403,7 +45403,7 @@
         <v>6</v>
       </c>
       <c r="O56" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P56" t="n">
         <v>0</v>
@@ -45511,7 +45511,7 @@
         <v>7</v>
       </c>
       <c r="O57" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="P57" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Zweihand-Grundkapazität eingerechnet: +1 bis Stahl / +2 ab Titan (36 B-Waffen)
- weapons.json v7.1: alle Zweihandwaffen (Hand = B) Stufe 1–6 erhalten
  +1 Grundkapazität bis Stufe 3 bzw. +2 ab Stufe 4 — mehr Kapazität, nicht
  mehr Slots; Ziel-Balance: Einhand allein < Zweihand < Einhand+Offhand
- Regel in meta.zweihand_kapazitaet_bonus dokumentiert; slot_templates
  bleiben die Einhand-Basis; Stufe-7-B-Waffen folgen mit Stellar-Kalibrierung
- Altlast bereinigt: slot_templates-Klasse 'Dolche' → 'Stichwaffen'
  (JSON + Excel-Sheet, analog zum stat_skalierung-Fix vom Audit)
- Excel Waffen-Sheet: 36 Kapazitätszellen aktualisiert
- GDD §5.3 (Einhand/Zweihand-Tabelle + Regel) und §11 aktualisiert
- CLAUDE.md: Kurzreferenz, Sitzungsstand (inkl. Default-Branch-Status:
  versehentlich zu 'Main' umbenannt statt gewechselt), nächste Schritte

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LMPve8W3NYqANspaTmaDDr
</commit_message>
<xml_diff>
--- a/data/itemliste_v7.xlsx
+++ b/data/itemliste_v7.xlsx
@@ -16717,7 +16717,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dolche</t>
+          <t>Stichwaffen</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -16766,7 +16766,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dolche</t>
+          <t>Stichwaffen</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -16815,7 +16815,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Dolche</t>
+          <t>Stichwaffen</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -16864,7 +16864,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Dolche</t>
+          <t>Stichwaffen</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -16913,7 +16913,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Dolche</t>
+          <t>Stichwaffen</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -16962,7 +16962,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Dolche</t>
+          <t>Stichwaffen</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -17011,7 +17011,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Dolche</t>
+          <t>Stichwaffen</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -20176,7 +20176,7 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P18" t="n">
         <v>1</v>
@@ -20283,7 +20283,7 @@
         </is>
       </c>
       <c r="O19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P19" t="n">
         <v>2</v>
@@ -20390,7 +20390,7 @@
         </is>
       </c>
       <c r="O20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P20" t="n">
         <v>3</v>
@@ -20497,7 +20497,7 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P21" t="n">
         <v>3</v>
@@ -20604,7 +20604,7 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P22" t="n">
         <v>3</v>
@@ -20711,7 +20711,7 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P23" t="n">
         <v>3</v>
@@ -21699,7 +21699,7 @@
         </is>
       </c>
       <c r="O33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P33" t="n">
         <v>1</v>
@@ -21806,7 +21806,7 @@
         </is>
       </c>
       <c r="O34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P34" t="n">
         <v>2</v>
@@ -21913,7 +21913,7 @@
         </is>
       </c>
       <c r="O35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P35" t="n">
         <v>3</v>
@@ -22020,7 +22020,7 @@
         </is>
       </c>
       <c r="O36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P36" t="n">
         <v>3</v>
@@ -22127,7 +22127,7 @@
         </is>
       </c>
       <c r="O37" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P37" t="n">
         <v>3</v>
@@ -22234,7 +22234,7 @@
         </is>
       </c>
       <c r="O38" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P38" t="n">
         <v>3</v>
@@ -23999,7 +23999,7 @@
         </is>
       </c>
       <c r="O56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P56" t="n">
         <v>1</v>
@@ -24106,7 +24106,7 @@
         </is>
       </c>
       <c r="O57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P57" t="n">
         <v>2</v>
@@ -24213,7 +24213,7 @@
         </is>
       </c>
       <c r="O58" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P58" t="n">
         <v>3</v>
@@ -24320,7 +24320,7 @@
         </is>
       </c>
       <c r="O59" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P59" t="n">
         <v>3</v>
@@ -24427,7 +24427,7 @@
         </is>
       </c>
       <c r="O60" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P60" t="n">
         <v>3</v>
@@ -24534,7 +24534,7 @@
         </is>
       </c>
       <c r="O61" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P61" t="n">
         <v>3</v>
@@ -26268,7 +26268,7 @@
         </is>
       </c>
       <c r="O78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P78" t="n">
         <v>1</v>
@@ -26377,7 +26377,7 @@
         </is>
       </c>
       <c r="O79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P79" t="n">
         <v>2</v>
@@ -26486,7 +26486,7 @@
         </is>
       </c>
       <c r="O80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P80" t="n">
         <v>3</v>
@@ -26595,7 +26595,7 @@
         </is>
       </c>
       <c r="O81" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P81" t="n">
         <v>3</v>
@@ -26704,7 +26704,7 @@
         </is>
       </c>
       <c r="O82" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P82" t="n">
         <v>3</v>
@@ -26813,7 +26813,7 @@
         </is>
       </c>
       <c r="O83" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P83" t="n">
         <v>3</v>
@@ -27788,7 +27788,7 @@
         </is>
       </c>
       <c r="O92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P92" t="n">
         <v>1</v>
@@ -27897,7 +27897,7 @@
         </is>
       </c>
       <c r="O93" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P93" t="n">
         <v>2</v>
@@ -28006,7 +28006,7 @@
         </is>
       </c>
       <c r="O94" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P94" t="n">
         <v>3</v>
@@ -28115,7 +28115,7 @@
         </is>
       </c>
       <c r="O95" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P95" t="n">
         <v>3</v>
@@ -28224,7 +28224,7 @@
         </is>
       </c>
       <c r="O96" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P96" t="n">
         <v>3</v>
@@ -28333,7 +28333,7 @@
         </is>
       </c>
       <c r="O97" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P97" t="n">
         <v>3</v>
@@ -28548,7 +28548,7 @@
         </is>
       </c>
       <c r="O99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P99" t="n">
         <v>1</v>
@@ -28657,7 +28657,7 @@
         </is>
       </c>
       <c r="O100" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P100" t="n">
         <v>2</v>
@@ -28766,7 +28766,7 @@
         </is>
       </c>
       <c r="O101" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P101" t="n">
         <v>3</v>
@@ -28875,7 +28875,7 @@
         </is>
       </c>
       <c r="O102" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P102" t="n">
         <v>3</v>
@@ -28984,7 +28984,7 @@
         </is>
       </c>
       <c r="O103" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P103" t="n">
         <v>3</v>
@@ -29093,7 +29093,7 @@
         </is>
       </c>
       <c r="O104" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P104" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Stellar-Kalibrierung: Stufe-7-Waffen final (weapons.json v8, GDD v0.15)
- Stufe-7-Werte: Prim 84/100/70, Sek analog; Kapazität +2 über Diamant
  (L4/L5-Signatur-Unlock), 5 Slots, Verfeinerung 3x, Verkauf 1000
- Stellar-Eigenarten (verstärkte Typ-Eigenart) + verstecktes
  Lichtresonanz-Flag (Story: durchdringt Schattenrüstung der Endfraktion)
- Sek-WID eingedampft: Jagd-/Langbogen auf Sek STR umgestellt (alle Bögen
  GES/STR), Hammer auf Körper-Rüstungs-Tier 3/5/7/10/13/17/23
- Zepter auf Zweihand (B) angeglichen, Kapazität 2/3/4/7/8/9/11
- Excel synchronisiert; Altlast Stat-Skalierung 'Dolche'->'Stichwaffen'

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cd4ivyUzihK6nnHF3i8Ag5
</commit_message>
<xml_diff>
--- a/data/itemliste_v7.xlsx
+++ b/data/itemliste_v7.xlsx
@@ -14567,7 +14567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14621,6 +14621,16 @@
           <t>Eigenart-Effekt</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Stellar-Eigenart ✦</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Stellar-Effekt</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -14663,6 +14673,16 @@
           <t>+15 % Rohschaden bei Frontalangriff</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Frontmann ✦</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>+25 % Rohschaden bei Frontalangriff</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -14705,6 +14725,16 @@
           <t>Markiert Ziel als 'Opfer' (1 gleichzeitig, springt weiter). Treffer auf Opfer: +20 % Schaden + 20 % Blutungsrisiko</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Erbarmungslos ✦</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Markiert Ziel als 'Opfer' (1 gleichzeitig, springt weiter). Treffer auf Opfer: +30 % Schaden + 30 % Blutungsrisiko</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -14747,6 +14777,16 @@
           <t>Treffen alle Ziele (Ziel + 2 Nachbarn): alle erhalten zusätzlich 30 % des Schadens</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Kollateralschaden ✦</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Treffen alle Ziele (Ziel + 2 Nachbarn): alle erhalten zusätzlich 50 % des Schadens</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -14789,6 +14829,16 @@
           <t>Treffer: Ziel verliert 1 MOB für den nächsten Zug</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Trägheit ✦</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Treffer: Ziel verliert 2 MOB für den nächsten Zug</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -14831,6 +14881,16 @@
           <t>Pusht Ziel 1 Feld zurück. Feld unbegehbar/belegt → 10 % max. LP Schaden + Straucheln (1 Runde, -50 % WID)</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Fliehkraft ✦</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Pusht Ziel 2 Felder zurück. Feld unbegehbar/belegt → 15 % max. LP Schaden + Straucheln (1 Runde, -50 % WID)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14873,6 +14933,16 @@
           <t>20 % des verursachten Schadens werden als Mana zurückerstattet</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Manavampir ✦</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>35 % des verursachten Schadens werden als Mana zurückerstattet</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -14915,6 +14985,16 @@
           <t>Nach Treffer: sofortige kostenlose Bewegung von 2 Feldern (1x pro Zug, mehrmals pro Runde möglich)</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Duellist ✦</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Nach Treffer: sofortige kostenlose Bewegung von 3 Feldern (1x pro Zug, mehrmals pro Runde möglich)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -14957,6 +15037,16 @@
           <t>Greift zweimal an — je 65 % Schaden pro Stich</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Dopplereffekt ✦</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Greift zweimal an — je 80 % Schaden pro Stich</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -14999,6 +15089,16 @@
           <t>Parieren triggert immer Gegenschlag; universell +20 % Parieren-Chance</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Fechtkunst ✦</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Parieren triggert immer Gegenschlag; universell +35 % Parieren-Chance</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -15041,6 +15141,16 @@
           <t>Backstab triggert immer Blutung; Backstabs haben +50 % Schaden</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Meuchelschlag ✦</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Backstab triggert immer Blutung; Backstabs haben +80 % Schaden</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -15070,7 +15180,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -15081,6 +15191,16 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>Deckt unsichtbare Gegner innerhalb der Bewegungsreichweite (MOB) auf</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Jagdinstinkt ✦</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Deckt unsichtbare Gegner innerhalb der Bewegungsreichweite (MOB) + 2 Felder auf</t>
         </is>
       </c>
     </row>
@@ -15125,6 +15245,16 @@
           <t>Kein Angriff letzten Zug → zweiter Bolzen geladen → nächster Angriff +50 % Schaden</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Techniker ✦</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Kein Angriff letzten Zug → zweiter Bolzen geladen → nächster Angriff +75 % Schaden</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -15154,7 +15284,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -15165,6 +15295,16 @@
       <c r="H14" t="inlineStr">
         <is>
           <t>Keine Bewegung letzten Zug → +30 % Schaden diesen Zug</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Heckenschütze ✦</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Keine Bewegung letzten Zug → +50 % Schaden diesen Zug</t>
         </is>
       </c>
     </row>
@@ -15209,6 +15349,16 @@
           <t>50 % Rüstungsdurchdringung (RD)</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Durchschlagskraft ✦</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>75 % Rüstungsdurchdringung (RD)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15251,6 +15401,16 @@
           <t>2 Züge ohne Schadenstreffer → Energieschild (Schutz) in Höhe des max. Mana</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Energiefaser ✦</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Bereits 1 Zug ohne Schadenstreffer → Energieschild (Schutz) in Höhe des max. Mana</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -15291,6 +15451,16 @@
       <c r="H17" t="inlineStr">
         <is>
           <t>Heilungen wirken zu Beginn des nächsten Zuges nochmals zu 20 %</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Segnung ✦</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Heilungen wirken zu Beginn des nächsten Zuges nochmals zu 35 %</t>
         </is>
       </c>
     </row>
@@ -15686,30 +15856,39 @@
           <t>Stellar</t>
         </is>
       </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
+          <t>Spezial</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>9</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -16020,30 +16199,39 @@
           <t>Stellar</t>
         </is>
       </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
+          <t>Spezial</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>9</v>
+      </c>
+      <c r="K15" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -16354,30 +16542,39 @@
           <t>Stellar</t>
         </is>
       </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
+          <t>Spezial</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>9</v>
+      </c>
+      <c r="K22" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -16688,30 +16885,39 @@
           <t>Stellar</t>
         </is>
       </c>
+      <c r="D29" t="n">
+        <v>5</v>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
+          <t>Spezial</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>9</v>
+      </c>
+      <c r="K29" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -17022,30 +17228,39 @@
           <t>Stellar</t>
         </is>
       </c>
+      <c r="D36" t="n">
+        <v>5</v>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
+          <t>Spezial</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>11</v>
+      </c>
+      <c r="K36" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="37">
@@ -17356,30 +17571,39 @@
           <t>Stellar</t>
         </is>
       </c>
+      <c r="D43" t="n">
+        <v>5</v>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
+          <t>Spezial</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>11</v>
+      </c>
+      <c r="K43" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="44">
@@ -17690,30 +17914,39 @@
           <t>Stellar</t>
         </is>
       </c>
+      <c r="D50" t="n">
+        <v>5</v>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
+          <t>Spezial</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>12</v>
+      </c>
+      <c r="K50" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="51">
@@ -17759,7 +17992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -17897,10 +18130,8 @@
       <c r="H2" t="n">
         <v>62</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I2" t="n">
+        <v>84</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -17925,10 +18156,8 @@
       <c r="P2" t="n">
         <v>38</v>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="Q2" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="3">
@@ -17960,10 +18189,8 @@
       <c r="H3" t="n">
         <v>74</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I3" t="n">
+        <v>100</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -17988,10 +18215,8 @@
       <c r="P3" t="n">
         <v>28</v>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="Q3" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="4">
@@ -18023,14 +18248,12 @@
       <c r="H4" t="n">
         <v>62</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I4" t="n">
+        <v>84</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>VIT/INT (typabh.)</t>
         </is>
       </c>
       <c r="K4" t="n">
@@ -18051,10 +18274,8 @@
       <c r="P4" t="n">
         <v>40</v>
       </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="Q4" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -18086,10 +18307,8 @@
       <c r="H5" t="n">
         <v>52</v>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I5" t="n">
+        <v>70</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -18114,16 +18333,14 @@
       <c r="P5" t="n">
         <v>40</v>
       </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="Q5" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dolche</t>
+          <t>Stichwaffen</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -18149,10 +18366,8 @@
       <c r="H6" t="n">
         <v>52</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I6" t="n">
+        <v>70</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -18177,10 +18392,8 @@
       <c r="P6" t="n">
         <v>52</v>
       </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="Q6" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="7">
@@ -18212,14 +18425,12 @@
       <c r="H7" t="n">
         <v>62</v>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I7" t="n">
+        <v>84</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="K7" t="n">
@@ -18240,10 +18451,8 @@
       <c r="P7" t="n">
         <v>28</v>
       </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="Q7" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="8">
@@ -18275,10 +18484,8 @@
       <c r="H8" t="n">
         <v>62</v>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="I8" t="n">
+        <v>84</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -18303,10 +18510,8 @@
       <c r="P8" t="n">
         <v>52</v>
       </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="Q8" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="9">
@@ -18384,6 +18589,79 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Kriegsgeräte — Sek-WID (nur Hammer, eingedampft 2026-07-04 = Körper-Rüstungs-Tier)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N10" t="n">
+        <v>10</v>
+      </c>
+      <c r="O10" t="n">
+        <v>13</v>
+      </c>
+      <c r="P10" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -19258,7 +19536,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Frontmann</t>
+          <t>Frontmann ✦</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -19267,38 +19545,38 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -19306,7 +19584,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -19314,7 +19592,7 @@
         </is>
       </c>
       <c r="T9" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="U9" t="n">
         <v>1</v>
@@ -19328,7 +19606,7 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="10">
@@ -20004,7 +20282,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Erbarmungslos</t>
+          <t>Erbarmungslos ✦</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -20013,38 +20291,38 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -20052,7 +20330,7 @@
         </is>
       </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -20060,7 +20338,7 @@
         </is>
       </c>
       <c r="T16" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="U16" t="n">
         <v>1</v>
@@ -20074,7 +20352,7 @@
         </is>
       </c>
       <c r="Y16" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="17">
@@ -20781,7 +21059,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Kollateralschaden</t>
+          <t>Kollateralschaden ✦</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -20790,38 +21068,38 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -20829,7 +21107,7 @@
         </is>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
@@ -20837,7 +21115,7 @@
         </is>
       </c>
       <c r="T24" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="U24" t="n">
         <v>1</v>
@@ -20851,7 +21129,7 @@
         </is>
       </c>
       <c r="Y24" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="25">
@@ -20972,7 +21250,7 @@
         </is>
       </c>
       <c r="T26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="U26" t="n">
         <v>1</v>
@@ -21079,7 +21357,7 @@
         </is>
       </c>
       <c r="T27" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U27" t="n">
         <v>1</v>
@@ -21186,7 +21464,7 @@
         </is>
       </c>
       <c r="T28" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="U28" t="n">
         <v>1</v>
@@ -21293,7 +21571,7 @@
         </is>
       </c>
       <c r="T29" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="U29" t="n">
         <v>1</v>
@@ -21400,7 +21678,7 @@
         </is>
       </c>
       <c r="T30" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="U30" t="n">
         <v>1</v>
@@ -21507,7 +21785,7 @@
         </is>
       </c>
       <c r="T31" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="U31" t="n">
         <v>1</v>
@@ -21558,7 +21836,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Trägheit</t>
+          <t>Trägheit ✦</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -21567,38 +21845,38 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O32" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P32" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -21606,7 +21884,7 @@
         </is>
       </c>
       <c r="R32" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
@@ -21614,7 +21892,7 @@
         </is>
       </c>
       <c r="T32" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="U32" t="n">
         <v>1</v>
@@ -21628,7 +21906,7 @@
         </is>
       </c>
       <c r="Y32" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="33">
@@ -22304,7 +22582,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Fliehkraft</t>
+          <t>Fliehkraft ✦</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -22313,38 +22591,38 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O39" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P39" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
@@ -22352,7 +22630,7 @@
         </is>
       </c>
       <c r="R39" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S39" t="inlineStr">
         <is>
@@ -22360,7 +22638,7 @@
         </is>
       </c>
       <c r="T39" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="U39" t="n">
         <v>1</v>
@@ -22374,7 +22652,7 @@
         </is>
       </c>
       <c r="Y39" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="40">
@@ -22445,7 +22723,7 @@
         </is>
       </c>
       <c r="O40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P40" t="n">
         <v>1</v>
@@ -22552,7 +22830,7 @@
         </is>
       </c>
       <c r="O41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P41" t="n">
         <v>2</v>
@@ -22659,7 +22937,7 @@
         </is>
       </c>
       <c r="O42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P42" t="n">
         <v>3</v>
@@ -22766,7 +23044,7 @@
         </is>
       </c>
       <c r="O43" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P43" t="n">
         <v>3</v>
@@ -22873,7 +23151,7 @@
         </is>
       </c>
       <c r="O44" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P44" t="n">
         <v>3</v>
@@ -22980,7 +23258,7 @@
         </is>
       </c>
       <c r="O45" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P45" t="n">
         <v>3</v>
@@ -23050,7 +23328,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Manavampir</t>
+          <t>Manavampir ✦</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -23059,38 +23337,38 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O46" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
@@ -23098,7 +23376,7 @@
         </is>
       </c>
       <c r="R46" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S46" t="inlineStr">
         <is>
@@ -23106,7 +23384,7 @@
         </is>
       </c>
       <c r="T46" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="U46" t="n">
         <v>1</v>
@@ -23120,7 +23398,7 @@
         </is>
       </c>
       <c r="Y46" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="47">
@@ -23827,7 +24105,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Duellist</t>
+          <t>Duellist ✦</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -23836,38 +24114,38 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O54" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P54" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
@@ -23875,7 +24153,7 @@
         </is>
       </c>
       <c r="R54" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="S54" t="inlineStr">
         <is>
@@ -23883,7 +24161,7 @@
         </is>
       </c>
       <c r="T54" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="U54" t="n">
         <v>1</v>
@@ -23897,7 +24175,7 @@
         </is>
       </c>
       <c r="Y54" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="55">
@@ -24604,7 +24882,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Dopplereffekt</t>
+          <t>Dopplereffekt ✦</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -24613,38 +24891,38 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O62" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="P62" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
@@ -24652,7 +24930,7 @@
         </is>
       </c>
       <c r="R62" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="S62" t="inlineStr">
         <is>
@@ -24660,7 +24938,7 @@
         </is>
       </c>
       <c r="T62" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="U62" t="n">
         <v>2</v>
@@ -24674,7 +24952,7 @@
         </is>
       </c>
       <c r="Y62" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="63">
@@ -25350,7 +25628,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Fechtkunst</t>
+          <t>Fechtkunst ✦</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -25359,38 +25637,38 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O69" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P69" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
@@ -25398,7 +25676,7 @@
         </is>
       </c>
       <c r="R69" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="S69" t="inlineStr">
         <is>
@@ -25406,7 +25684,7 @@
         </is>
       </c>
       <c r="T69" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="U69" t="n">
         <v>1</v>
@@ -25420,7 +25698,7 @@
         </is>
       </c>
       <c r="Y69" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="70">
@@ -26096,7 +26374,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Meuchelschlag</t>
+          <t>Meuchelschlag ✦</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -26105,38 +26383,38 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O76" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P76" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
@@ -26144,7 +26422,7 @@
         </is>
       </c>
       <c r="R76" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="S76" t="inlineStr">
         <is>
@@ -26152,7 +26430,7 @@
         </is>
       </c>
       <c r="T76" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="U76" t="n">
         <v>1</v>
@@ -26166,7 +26444,7 @@
         </is>
       </c>
       <c r="Y76" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="77">
@@ -26283,7 +26561,7 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T78" t="n">
@@ -26392,7 +26670,7 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T79" t="n">
@@ -26501,7 +26779,7 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T80" t="n">
@@ -26610,7 +26888,7 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T81" t="n">
@@ -26719,7 +26997,7 @@
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T82" t="n">
@@ -26828,7 +27106,7 @@
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T83" t="n">
@@ -26885,7 +27163,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Jagdinstinkt</t>
+          <t>Jagdinstinkt ✦</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -26894,38 +27172,38 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O84" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="P84" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
@@ -26933,15 +27211,15 @@
         </is>
       </c>
       <c r="R84" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T84" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="U84" t="n">
         <v>1</v>
@@ -26957,7 +27235,7 @@
         </is>
       </c>
       <c r="Y84" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="85">
@@ -27645,7 +27923,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Techniker</t>
+          <t>Techniker ✦</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -27654,38 +27932,38 @@
         </is>
       </c>
       <c r="I91" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O91" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P91" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
@@ -27693,7 +27971,7 @@
         </is>
       </c>
       <c r="R91" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S91" t="inlineStr">
         <is>
@@ -27701,7 +27979,7 @@
         </is>
       </c>
       <c r="T91" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="U91" t="n">
         <v>1</v>
@@ -27717,7 +27995,7 @@
         </is>
       </c>
       <c r="Y91" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="92">
@@ -27803,7 +28081,7 @@
       </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T92" t="n">
@@ -27912,7 +28190,7 @@
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T93" t="n">
@@ -28021,7 +28299,7 @@
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T94" t="n">
@@ -28130,7 +28408,7 @@
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T95" t="n">
@@ -28239,7 +28517,7 @@
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T96" t="n">
@@ -28348,7 +28626,7 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T97" t="n">
@@ -28405,7 +28683,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Heckenschütze</t>
+          <t>Heckenschütze ✦</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -28414,38 +28692,38 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O98" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="P98" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
@@ -28453,15 +28731,15 @@
         </is>
       </c>
       <c r="R98" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>WID</t>
+          <t>STR</t>
         </is>
       </c>
       <c r="T98" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="U98" t="n">
         <v>1</v>
@@ -28477,7 +28755,7 @@
         </is>
       </c>
       <c r="Y98" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="99">
@@ -29165,7 +29443,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Durchschlagskraft</t>
+          <t>Durchschlagskraft ✦</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -29174,38 +29452,38 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O105" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="P105" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q105" t="inlineStr">
         <is>
@@ -29213,7 +29491,7 @@
         </is>
       </c>
       <c r="R105" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S105" t="inlineStr">
         <is>
@@ -29221,7 +29499,7 @@
         </is>
       </c>
       <c r="T105" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="U105" t="n">
         <v>1</v>
@@ -29237,7 +29515,7 @@
         </is>
       </c>
       <c r="Y105" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="106">
@@ -29944,7 +30222,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Energiefaser</t>
+          <t>Energiefaser ✦</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -29953,38 +30231,38 @@
         </is>
       </c>
       <c r="I113" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O113" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P113" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
@@ -29992,7 +30270,7 @@
         </is>
       </c>
       <c r="R113" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S113" t="inlineStr">
         <is>
@@ -30000,7 +30278,7 @@
         </is>
       </c>
       <c r="T113" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="U113" t="n">
         <v>1</v>
@@ -30014,7 +30292,7 @@
         </is>
       </c>
       <c r="Y113" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="114">
@@ -30690,7 +30968,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Segnung</t>
+          <t>Segnung ✦</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -30699,38 +30977,38 @@
         </is>
       </c>
       <c r="I120" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Aktiv</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Passiv</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Reaktiv</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Mod.</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Spezial</t>
         </is>
       </c>
       <c r="O120" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P120" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q120" t="inlineStr">
         <is>
@@ -30738,7 +31016,7 @@
         </is>
       </c>
       <c r="R120" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="S120" t="inlineStr">
         <is>
@@ -30746,7 +31024,7 @@
         </is>
       </c>
       <c r="T120" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="U120" t="n">
         <v>1</v>
@@ -30760,7 +31038,7 @@
         </is>
       </c>
       <c r="Y120" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Schadenstyp-Audit: Rohschaden-Formel-Klärung, Kriegsgeräte-Neuordnung, Statuseffekt-Harmonisierung (GDD v0.19)
- Magisch-Rohschaden gilt jetzt explizit reichweitenunabhängig (deckt Zauberstab/Energiesphäre ab)
- Kriegsgeräte neu geordnet: Hammer/Rammbock Prim WID + Sek STR, Zepter Prim WIL + Sek WID (statt INT)
- Brennen/In Brand gesteckt -> Hitzeschaden, Vergiftet/Gift/Giftnebel -> Terraschaden
- "Zauberschaden"-Boni wirken auf Rohschaden vor dem Elementar-Split
- weapons.json (stat_skalierung, waffentypen, Items) und itemliste_v7.xlsx synchronisiert
</commit_message>
<xml_diff>
--- a/data/itemliste_v7.xlsx
+++ b/data/itemliste_v7.xlsx
@@ -14811,12 +14811,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>STR</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>WID</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -14863,12 +14863,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>STR</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>VIT</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -14920,7 +14920,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>WID</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -17992,7 +17992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -18227,55 +18227,83 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>STR</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F4" t="n">
-        <v>32</v>
-      </c>
-      <c r="G4" t="n">
-        <v>45</v>
-      </c>
-      <c r="H4" t="n">
-        <v>62</v>
-      </c>
-      <c r="I4" t="n">
-        <v>84</v>
+          <t>WID/WIL (typabh., s. u.)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>VIT/INT (typabh.)</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L4" t="n">
-        <v>9</v>
-      </c>
-      <c r="M4" t="n">
-        <v>14</v>
-      </c>
-      <c r="N4" t="n">
-        <v>20</v>
-      </c>
-      <c r="O4" t="n">
-        <v>28</v>
-      </c>
-      <c r="P4" t="n">
-        <v>40</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>54</v>
+          <t>STR/WID (typabh., s. u.)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -18594,73 +18622,118 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kriegsgeräte — Sek-WID (nur Hammer, eingedampft 2026-07-04 = Körper-Rüstungs-Tier)</t>
+          <t>Kriegsgeräte — Hammer &amp; Rammbock: Prim WID / Sek STR (physische Zäh-Bruiser, 2026-07-07)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" t="n">
+        <v>13</v>
+      </c>
+      <c r="H10" t="n">
+        <v>17</v>
+      </c>
+      <c r="I10" t="n">
+        <v>23</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
+          <t>STR</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" t="n">
+        <v>9</v>
+      </c>
+      <c r="M10" t="n">
+        <v>14</v>
+      </c>
+      <c r="N10" t="n">
+        <v>20</v>
+      </c>
+      <c r="O10" t="n">
+        <v>28</v>
+      </c>
+      <c r="P10" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kriegsgeräte — Zepter: Prim WIL / Sek WID (Magie-Nahkämpfer, unverändert Rohschaden-relevant, 2026-07-07)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>WIL</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" t="n">
+        <v>22</v>
+      </c>
+      <c r="F11" t="n">
+        <v>32</v>
+      </c>
+      <c r="G11" t="n">
+        <v>45</v>
+      </c>
+      <c r="H11" t="n">
+        <v>62</v>
+      </c>
+      <c r="I11" t="n">
+        <v>84</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>WID</t>
         </is>
       </c>
-      <c r="K10" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" t="n">
+      <c r="K11" t="n">
+        <v>3</v>
+      </c>
+      <c r="L11" t="n">
         <v>5</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M11" t="n">
         <v>7</v>
       </c>
-      <c r="N10" t="n">
+      <c r="N11" t="n">
         <v>10</v>
       </c>
-      <c r="O10" t="n">
+      <c r="O11" t="n">
         <v>13</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P11" t="n">
         <v>17</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="Q11" t="n">
         <v>23</v>
       </c>
     </row>
@@ -21238,19 +21311,19 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R26" t="n">
+        <v>3</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
           <t>STR</t>
         </is>
       </c>
-      <c r="R26" t="n">
-        <v>10</v>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>WID</t>
-        </is>
-      </c>
       <c r="T26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="U26" t="n">
         <v>1</v>
@@ -21345,19 +21418,19 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R27" t="n">
+        <v>5</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
           <t>STR</t>
         </is>
       </c>
-      <c r="R27" t="n">
-        <v>15</v>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>WID</t>
-        </is>
-      </c>
       <c r="T27" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="U27" t="n">
         <v>1</v>
@@ -21452,19 +21525,19 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R28" t="n">
+        <v>7</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
           <t>STR</t>
         </is>
       </c>
-      <c r="R28" t="n">
-        <v>22</v>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>WID</t>
-        </is>
-      </c>
       <c r="T28" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="U28" t="n">
         <v>1</v>
@@ -21559,19 +21632,19 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R29" t="n">
+        <v>10</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
           <t>STR</t>
         </is>
       </c>
-      <c r="R29" t="n">
-        <v>32</v>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>WID</t>
-        </is>
-      </c>
       <c r="T29" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="U29" t="n">
         <v>1</v>
@@ -21666,19 +21739,19 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R30" t="n">
+        <v>13</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
           <t>STR</t>
         </is>
       </c>
-      <c r="R30" t="n">
-        <v>45</v>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>WID</t>
-        </is>
-      </c>
       <c r="T30" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="U30" t="n">
         <v>1</v>
@@ -21773,19 +21846,19 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R31" t="n">
+        <v>17</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
           <t>STR</t>
         </is>
       </c>
-      <c r="R31" t="n">
-        <v>62</v>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>WID</t>
-        </is>
-      </c>
       <c r="T31" t="n">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="U31" t="n">
         <v>1</v>
@@ -21880,19 +21953,19 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R32" t="n">
+        <v>23</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
           <t>STR</t>
         </is>
       </c>
-      <c r="R32" t="n">
-        <v>84</v>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>WID</t>
-        </is>
-      </c>
       <c r="T32" t="n">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="U32" t="n">
         <v>1</v>
@@ -21984,15 +22057,15 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R33" t="n">
+        <v>3</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
           <t>STR</t>
-        </is>
-      </c>
-      <c r="R33" t="n">
-        <v>10</v>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>VIT</t>
         </is>
       </c>
       <c r="T33" t="n">
@@ -22091,15 +22164,15 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R34" t="n">
+        <v>5</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
           <t>STR</t>
-        </is>
-      </c>
-      <c r="R34" t="n">
-        <v>15</v>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>VIT</t>
         </is>
       </c>
       <c r="T34" t="n">
@@ -22198,15 +22271,15 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>7</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
           <t>STR</t>
-        </is>
-      </c>
-      <c r="R35" t="n">
-        <v>22</v>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>VIT</t>
         </is>
       </c>
       <c r="T35" t="n">
@@ -22305,15 +22378,15 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R36" t="n">
+        <v>10</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
           <t>STR</t>
-        </is>
-      </c>
-      <c r="R36" t="n">
-        <v>32</v>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>VIT</t>
         </is>
       </c>
       <c r="T36" t="n">
@@ -22412,15 +22485,15 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>13</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
           <t>STR</t>
-        </is>
-      </c>
-      <c r="R37" t="n">
-        <v>45</v>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>VIT</t>
         </is>
       </c>
       <c r="T37" t="n">
@@ -22519,15 +22592,15 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R38" t="n">
+        <v>17</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
           <t>STR</t>
-        </is>
-      </c>
-      <c r="R38" t="n">
-        <v>62</v>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>VIT</t>
         </is>
       </c>
       <c r="T38" t="n">
@@ -22626,15 +22699,15 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
+          <t>WID</t>
+        </is>
+      </c>
+      <c r="R39" t="n">
+        <v>23</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
           <t>STR</t>
-        </is>
-      </c>
-      <c r="R39" t="n">
-        <v>84</v>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>VIT</t>
         </is>
       </c>
       <c r="T39" t="n">
@@ -22738,11 +22811,11 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>WID</t>
         </is>
       </c>
       <c r="T40" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="U40" t="n">
         <v>1</v>
@@ -22845,11 +22918,11 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>WID</t>
         </is>
       </c>
       <c r="T41" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U41" t="n">
         <v>1</v>
@@ -22952,11 +23025,11 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>WID</t>
         </is>
       </c>
       <c r="T42" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="U42" t="n">
         <v>1</v>
@@ -23059,11 +23132,11 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>WID</t>
         </is>
       </c>
       <c r="T43" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="U43" t="n">
         <v>1</v>
@@ -23166,11 +23239,11 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>WID</t>
         </is>
       </c>
       <c r="T44" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="U44" t="n">
         <v>1</v>
@@ -23273,11 +23346,11 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>WID</t>
         </is>
       </c>
       <c r="T45" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="U45" t="n">
         <v>1</v>
@@ -23380,11 +23453,11 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>WID</t>
         </is>
       </c>
       <c r="T46" t="n">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="U46" t="n">
         <v>1</v>

</xml_diff>